<commit_message>
Expand references to 5-6 sources per row in workbook and reference doc
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014pjai2kqP2WpfNbADBXAaM
</commit_message>
<xml_diff>
--- a/Active ETF scoping - references filled.xlsx
+++ b/Active ETF scoping - references filled.xlsx
@@ -496,7 +496,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="345" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t>What exactly is an active ETF? What are the mechanics?</t>
@@ -524,7 +524,11 @@
 3. How ETF shares are bought/sold and the mechanics of NAV, bid/ask spread and liquidity (creation/redemption, market makers) – State Street Global Advisors
 https://www.ssga.com/us/en/intermediary/insights/master-the-mechanics-of-etf-trading
 4. Technical reference on ETF mechanics (creation/redemption, premiums/discounts, trading and liquidity) – CFA Institute
-https://www.cfainstitute.org/insights/professional-learning/refresher-readings/2026/exchange-traded-funds-mechanics-applications</t>
+https://www.cfainstitute.org/insights/professional-learning/refresher-readings/2026/exchange-traded-funds-mechanics-applications
+5. Regulator's plain-English definition of active management and what it means for investors – U.S. SEC, Investor.gov glossary
+https://www.investor.gov/introduction-investing/investing-basics/glossary/active-fund-actively-managed-fund
+6. How active management is delivered inside the ETF vehicle – T. Rowe Price, “How to Gain the Benefits of Active Management in an Exchange-Traded Fund”
+https://www.troweprice.com/en/us/insights/gain-benefits-of-active-management-in-an-exchange-traded-fund</t>
         </is>
       </c>
     </row>
@@ -557,7 +561,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="255" customHeight="1">
+    <row r="6" ht="409" customHeight="1">
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>How is an active ETF different from an active fund?</t>
@@ -581,11 +585,15 @@
 2. Why the ETF wrapper is generally more tax-efficient than a mutual fund (in-kind creation/redemption) – Fidelity
 https://www.fidelity.com/learning-center/investment-products/etf/etfs-tax-efficiency
 3. Data point: only ~9% of active ETFs distributed a capital gain vs ~53% of active mutual funds – State Street Global Advisors
-https://www.ssga.com/us/en/individual/insights/tax-efficiency-is-structural-etfs-continue-to-issue-fewer-capital-gains-than-mutual-funds</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="255" customHeight="1">
+https://www.ssga.com/us/en/individual/insights/tax-efficiency-is-structural-etfs-continue-to-issue-fewer-capital-gains-than-mutual-funds
+4. Manager's view on what changes (and what doesn't) when an active strategy moves from a mutual fund to an ETF wrapper – T. Rowe Price, “Active ETFs Designed to Outperform”
+https://www.troweprice.com/financial-intermediary/us/en/insights/articles/2021/q3/active-etfs-designed-to-outperform.html
+5. Primer on how active ETFs work in much the same way as actively managed mutual funds, plus wrapper advantages – Hilton Capital Management, “Understanding Active ETFs”
+https://www.hiltoncapitalmanagement.com/understanding-active-etfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="409" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>How is an active ETF different from a passive ETF?</t>
@@ -611,11 +619,15 @@
 2. The cost trade-off: higher fees mean active ETFs must clear a higher bar, with fee/performance data – Morningstar
 https://www.morningstar.com/funds/active-versus-passive-etfs-why-lower-fees-still-win
 3. How the active/passive distinction is becoming a spectrum (systematic active, factor strategies) – Morningstar
-https://www.morningstar.com/funds/how-line-between-active-passive-etfs-is-blurring</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="330" customHeight="1">
+https://www.morningstar.com/funds/how-line-between-active-passive-etfs-is-blurring
+4. What active and passive ETFs share (the wrapper) and where they diverge (the strategy) – J.P. Morgan Asset Management, “ETFs Explained #1: Similarities of Active and Passive ETFs”
+https://am.jpmorgan.com/au/en/asset-management/adv/insights/investment-ideas/similarities-etfs/
+5. Balanced overview of the active vs passive trade-offs from the leading indexing provider – Vanguard, “Passive vs Active Investing: What's the Difference?”
+https://www3.vanguard.com.au/personal/learn/investment-options/active-vs-passive-investing</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="409" customHeight="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>What are some risks or limitations of active ETFs?</t>
@@ -643,7 +655,11 @@
 3. Liquidity and trading concerns: price returns of some active ETFs lag their NAV returns because of trading frictions – Morningstar
 https://www.morningstar.com/funds/you-might-not-always-get-returns-your-active-etf-earned
 4. Trading costs beyond the expense ratio (bid/ask spreads on active ETFs) – Morningstar
-https://www.morningstar.com/funds/your-active-etf-is-cheap-your-trade-might-not-be</t>
+https://www.morningstar.com/funds/your-active-etf-is-cheap-your-trade-might-not-be
+5. Whether active ETFs are inherently riskier than passive ETFs (risk depends on the underlying investments) – J.P. Morgan Asset Management, “Myth Busting #1”
+https://am.jpmorgan.com/sg/en/asset-management/adv/insights/portfolio-insights/etf-perspectives/active-etf-manual/myth-busting-active-etf-risks/
+6. Regulator's note that active funds typically carry higher costs and may underperform their index – U.S. SEC, Investor.gov
+https://www.investor.gov/introduction-investing/investing-basics/glossary/active-fund-actively-managed-fund</t>
         </is>
       </c>
     </row>
@@ -676,7 +692,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="255" customHeight="1">
+    <row r="12" ht="409" customHeight="1">
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Why would I use an active ETF? Which strategies should it be used for?</t>
@@ -701,11 +717,15 @@
 2. Whitepaper on active ETF categories and the manager's role in adding value – iShares/BlackRock, “Decoding Active ETFs”
 https://www.ishares.com/us/literature/whitepaper/decoding-active-etfs.pdf
 3. The case for active ETFs now – market conditions and strategy fit – Fidelity Institutional, “Why Active ETFs, Why Now?”
-https://institutional.fidelity.com/advisors/insights/topics/investing-ideas/why-active-etfs-why-now</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="255" customHeight="1">
+https://institutional.fidelity.com/advisors/insights/topics/investing-ideas/why-active-etfs-why-now
+4. What advisors need to know about the rapid rise of active ETFs (42% of Q1 2026 net inflows) and where they fit – VettaFi via Advisor Perspectives
+https://www.advisorperspectives.com/commentaries/2026/02/11/what-advisors-need-to-know-about-the-rapid-rise-of-active-etfs
+5. Where manager judgement is designed to add value over an index – T. Rowe Price, “Active ETFs Designed to Outperform”
+https://www.troweprice.com/financial-intermediary/us/en/insights/articles/2021/q3/active-etfs-designed-to-outperform.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="409" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Which clients are suitable for an active ETF?</t>
@@ -731,11 +751,15 @@
 2. Which active ETF categories advisors actually use and the client needs they map to (income, cash management, tax-efficient core) – The Daily Upside (Advisor)
 https://www.thedailyupside.com/advisor/investing-strategies/here-are-the-top-active-etfs-used-by-advisors/
 3. When advisors do (and don't) recommend active ETFs to clients – etf.com Advisor Center
-https://www.etf.com/sections/advisor-center/active-etf-financial-advisor-jpst-jaaa</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="345" customHeight="1">
+https://www.etf.com/sections/advisor-center/active-etf-financial-advisor-jpst-jaaa
+4. Advisor demand signal: 88% of advisors somewhat/very likely to increase active fixed income ETF allocations – VettaFi via Advisor Perspectives, “How Advisors Are Rewiring Fixed Income Portfolios”
+https://www.advisorperspectives.com/commentaries/2026/04/10/how-advisors-are-rewiring-fixed-income-portfolios
+5. Matching more conservative active ETF products to more conservative client profiles – ETF Trends, “Capital Group's Newer Active ETFs Offer More Conservative Approach”
+https://www.etftrends.com/capital-groups-newer-active-etfs-offer-more-conservative-approach/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="409" customHeight="1">
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t>How do I evaluate an active ETF that is right for my client?</t>
@@ -762,11 +786,15 @@
 3. Qualitative + quantitative evaluation of active ETFs (philosophy, team, liquidity, spreads) – Goldman Sachs Asset Management
 https://am.gs.com/en-us/advisors/insights/article/2026/active-etf-due-diligence-combination-of-art-and-science
 4. Step-by-step checklist for comparing active ETF options across a peer group – Mackenzie Investments
-https://www.mackenzieinvestments.com/en/investments/by-type/etfs/etf-articles/your-step-by-step-guide-to-active-etf-due-diligence</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="270" customHeight="1">
+https://www.mackenzieinvestments.com/en/investments/by-type/etfs/etf-articles/your-step-by-step-guide-to-active-etf-due-diligence
+5. General ETF due diligence checklist (costs, liquidity, structure, issuer strength) – State Street Global Advisors
+https://www.ssga.com/us/en/intermediary/insights/a-etf-due-diligence-checklist
+6. Issuer framework for evaluating active ETFs across the peer group (PDF) – J.P. Morgan Asset Management, “Evaluating Active ETFs”
+https://am.jpmorgan.com/content/dam/jpm-am-aem/asiapacific/au/en/etf/evaluating-active-etf.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="375" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>How do I approach ETFs by client type?</t>
@@ -791,7 +819,9 @@
 2. Adapting communication style to client personality types when presenting recommendations – Brighthouse Financial, “A Guide to Speaking Your Client's Language”
 https://www.brighthousefinancial.com/content/dam/brighthouse-financial/protected/pdfs/shield/Guide-Speaking-Clients-Language.pdf
 3. Understanding the beliefs and concerns behind client resistance before responding – Hartford Funds
-https://www.hartfordfunds.com/insights/investor-insight/investor-behavior/your-money-story/how-to-respond-when-a-client-resists-recommendations.html</t>
+https://www.hartfordfunds.com/insights/investor-insight/investor-behavior/your-money-story/how-to-respond-when-a-client-resists-recommendations.html
+4. The four most common misconceptions advisors will meet across client types, with rebuttals – J.P. Morgan Asset Management, “Active ETF Investing: Four Myths Debunked”
+https://am.jpmorgan.com/ca/en/asset-management/adv/funds/etf-perspectives/active-etf-investing-myths/</t>
         </is>
       </c>
     </row>
@@ -824,7 +854,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="270" customHeight="1">
+    <row r="19" ht="409" customHeight="1">
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>How do I introduce active ETFs into a client conversation?</t>
@@ -848,11 +878,15 @@
 2. Tools and talking points for structuring client conversations around goals and market events – Russell Investments, Client Conversation Center
 https://russellinvestments.com/content/ri/us/en/financial-professional/tools-and-education/business-solutions/client-conversation-center.html
 3. Framing the active ETF opportunity with clients (growth of the category and where it fits) – AllianceBernstein
-https://www.alliancebernstein.com/us/en-us/investments/etfs/etf-insights/actively-managed-etfs-are-on-the-move.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="315" customHeight="1">
+https://www.alliancebernstein.com/us/en-us/investments/etfs/etf-insights/actively-managed-etfs-are-on-the-move.html
+4. Current conversation hook: active ETFs took 42% of Q1 2026 net inflows and what that means for client portfolios – VettaFi via Advisor Perspectives
+https://www.advisorperspectives.com/commentaries/2026/02/11/what-advisors-need-to-know-about-the-rapid-rise-of-active-etfs
+5. How one issuer coaches advisors to pair active ETFs with client goals (accumulation vs decumulation) – ETF Database, “How Capital Group Shifted the Active ETF Playbook”
+https://etfdb.com/equity-etf-content-hub/capital-group-shifted-active-playbook/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="409" customHeight="1">
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t>What questions or objections can I expect from clients?</t>
@@ -882,11 +916,15 @@
 3. “Can active ETFs really outperform?” – whether outperformance persists – S&amp;P Dow Jones Indices, SPIVA Persistence Scorecard
 https://www.spglobal.com/spdji/en/spiva/article/us-persistence-scorecard/
 4. “Why should I pay more?” – fee differentials between active and passive ETFs – Morningstar
-https://www.morningstar.com/funds/active-versus-passive-etfs-why-lower-fees-still-win</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="270" customHeight="1">
+https://www.morningstar.com/funds/active-versus-passive-etfs-why-lower-fees-still-win
+5. “Aren't active ETFs riskier than passive ones?” – risk depends on the underlying investments, not the management style – J.P. Morgan Asset Management, “Myth Busting #1”
+https://am.jpmorgan.com/sg/en/asset-management/adv/insights/portfolio-insights/etf-perspectives/active-etf-manual/myth-busting-active-etf-risks/
+6. The four most common active ETF objections in one place, each answered – J.P. Morgan Asset Management, “Active ETF Investing: Four Myths Debunked”
+https://am.jpmorgan.com/ca/en/asset-management/adv/funds/etf-perspectives/active-etf-investing-myths/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="409" customHeight="1">
       <c r="B21" s="3" t="inlineStr">
         <is>
           <t>How do I respond to client objections?</t>
@@ -912,7 +950,11 @@
 2. A repeatable framework for handling clients who reject recommendations while keeping the discussion on goals – Kitces.com
 https://www.kitces.com/blog/163-michael-kitces-carl-richards-client-advice-implementation-recommendation-communication/
 3. Proof points for the active ETF wrapper vs active mutual funds and passive index funds (cost, tax efficiency, flexibility) – Fidelity Institutional
-https://institutional.fidelity.com/advisors/investment-solutions/strategies/active-etfs</t>
+https://institutional.fidelity.com/advisors/investment-solutions/strategies/active-etfs
+4. Ready-made rebuttals to the four most common objections (risk, liquidity, cost, performance) – J.P. Morgan Asset Management, “Active ETF Investing: Four Myths Debunked”
+https://am.jpmorgan.com/ca/en/asset-management/adv/funds/etf-perspectives/active-etf-investing-myths/
+5. Proof points vs passive: where active ETFs are designed to outperform and the evidence behind it – T. Rowe Price
+https://www.troweprice.com/financial-intermediary/us/en/insights/articles/2021/q3/active-etfs-designed-to-outperform.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rework references: Capital Group sources, internal RiF deck citations, curated externals
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014pjai2kqP2WpfNbADBXAaM
</commit_message>
<xml_diff>
--- a/Active ETF scoping - references filled.xlsx
+++ b/Active ETF scoping - references filled.xlsx
@@ -464,7 +464,7 @@
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="85" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -517,22 +517,26 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>1. What an actively managed ETF is, how active management works inside the ETF wrapper, and potential benefits/costs – Fidelity
-https://www.fidelity.com/learning-center/investment-products/etf/types-of-etfs-actively-managed
-2. Investor-level guide to what active ETFs are and how they differ from index ETFs – etf.com
-https://www.etf.com/sections/etf-basics/what-are-active-etfs-investing-guide
-3. How ETF shares are bought/sold and the mechanics of NAV, bid/ask spread and liquidity (creation/redemption, market makers) – State Street Global Advisors
+          <t>[Capital Group]
+1. “What is an ETF?” — definition, how shares trade at market price vs NAV
+https://www.capitalgroup.com/ria/investments/exchange-traded-funds/resources/what-is-an-etf.html
+2. ETF investing guide — mechanics, buying/selling, trading best practices (limit orders)
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/ETF-investing-guide.html
+3. ETF Insights &amp; Resources hub — full advisor education library on active ETFs
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources.html
+[Internal research]
+4. How fund selectors actually define an active ETF (key features, tracking-error spectrum) — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Section 5 “Defining active ETFs”
+[External]
+5. ETF trading mechanics: NAV, bid/ask spread, liquidity, creation/redemption — State Street Global Advisors
 https://www.ssga.com/us/en/intermediary/insights/master-the-mechanics-of-etf-trading
-4. Technical reference on ETF mechanics (creation/redemption, premiums/discounts, trading and liquidity) – CFA Institute
+6. Technical reference on ETF mechanics and applications — CFA Institute
 https://www.cfainstitute.org/insights/professional-learning/refresher-readings/2026/exchange-traded-funds-mechanics-applications
-5. Regulator's plain-English definition of active management and what it means for investors – U.S. SEC, Investor.gov glossary
-https://www.investor.gov/introduction-investing/investing-basics/glossary/active-fund-actively-managed-fund
-6. How active management is delivered inside the ETF vehicle – T. Rowe Price, “How to Gain the Benefits of Active Management in an Exchange-Traded Fund”
-https://www.troweprice.com/en/us/insights/gain-benefits-of-active-management-in-an-exchange-traded-fund</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="255" customHeight="1">
+7. What an actively managed ETF is and how it works — Fidelity
+https://www.fidelity.com/learning-center/investment-products/etf/types-of-etfs-actively-managed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="409" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Why have active ETFs become so widespread?</t>
@@ -552,11 +556,17 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>1. Younger investors choosing to work with advisors who include active ETFs in their investment approach
+          <t>[Capital Group]
+1. Active ETF solutions landing — Capital Group's positioning of the category's growth
+https://www.capitalgroup.com/active-etf
+[Internal research]
+2. ETF timeline: first active ETF 2010 → $1 trillion in active ETFs globally by 2024; US vs Europe flows; Rogers adoption curve showing active ETFs at the early-adopter stage — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Sections 1–2, slides 6–9
+[External]
+3. Younger investors choosing to work with advisors who include active ETFs in their investment approach — InvestmentNews
 https://www.investmentnews.com/practice-management/could-active-etfs-be-a-client-acquisition-magnet/259875
-2. Clients increasingly wants to understand what they own – Active ETFs provide transparency and flexibility
+4. Clients increasingly want to understand what they own — active ETFs provide transparency and flexibility — RFI Global
 https://rfi.global/planning-for-2026-five-us-consumer-trends-financial-institutions-cant-ignore/
-3. Increasing global adoption – active ETF flows increasing at a greater rate vs passive – BlackRock, “Active ETFs: Accelerating Adoption”
+5. Increasing global adoption — active ETF flows growing at a greater rate vs passive — BlackRock
 https://www.blackrock.com/us/financial-professionals/insights/exploring-active-etfs</t>
         </is>
       </c>
@@ -580,16 +590,22 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>1. Side-by-side comparison of ETFs vs mutual funds (trading, minimums, costs, use cases) – Charles Schwab
+          <t>[Capital Group]
+1. “ETF tax efficiency, explained” — video on externalization and in-kind redemption vs mutual funds
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/etf-tax-efficiency-explained.html
+2. “Mythbusted: Active ETFs can be as tax efficient as passive ETFs” — CG's own capital-gains record as proof the wrapper (not passive management) drives tax efficiency
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/mythbusted-CG-capital-gains.html
+3. “Tax-efficient investing with ETFs” — wrapper-level differences that matter to clients
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/tax-efficiency.html
+[Internal research]
+4. ~50% of ETF users expect ETFs to be preferred to, or replace, mutual funds; only 7% expect mutual funds preferred; ETF-vs-mutual-fund preference by market and client type — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Section 3 “Future expectations”, slides 18, 37–39
+[External]
+5. Side-by-side ETF vs mutual fund comparison (trading, minimums, costs, use cases) — Charles Schwab
 https://www.schwab.com/learn/story/etf-vs-mutual-fund-it-depends-on-your-strategy
-2. Why the ETF wrapper is generally more tax-efficient than a mutual fund (in-kind creation/redemption) – Fidelity
-https://www.fidelity.com/learning-center/investment-products/etf/etfs-tax-efficiency
-3. Data point: only ~9% of active ETFs distributed a capital gain vs ~53% of active mutual funds – State Street Global Advisors
+6. Data point: only ~9% of active ETFs distributed a capital gain vs ~53% of active mutual funds — State Street Global Advisors
 https://www.ssga.com/us/en/individual/insights/tax-efficiency-is-structural-etfs-continue-to-issue-fewer-capital-gains-than-mutual-funds
-4. Manager's view on what changes (and what doesn't) when an active strategy moves from a mutual fund to an ETF wrapper – T. Rowe Price, “Active ETFs Designed to Outperform”
-https://www.troweprice.com/financial-intermediary/us/en/insights/articles/2021/q3/active-etfs-designed-to-outperform.html
-5. Primer on how active ETFs work in much the same way as actively managed mutual funds, plus wrapper advantages – Hilton Capital Management, “Understanding Active ETFs”
-https://www.hiltoncapitalmanagement.com/understanding-active-etfs</t>
+7. What changes (and what doesn't) when an active strategy moves from a mutual fund to an ETF wrapper — T. Rowe Price
+https://www.troweprice.com/financial-intermediary/us/en/insights/articles/2021/q3/active-etfs-designed-to-outperform.html</t>
         </is>
       </c>
     </row>
@@ -614,16 +630,18 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>1. The case for active ETFs vs index-tracking ETFs (similarities, differences, potential for outperformance) – Aberdeen Investments, “Know Your ETFs: Why Active”
+          <t>[Capital Group]
+1. “The benefits of active ETFs” — potential for better-than-market outcomes and downside protection vs index tracking
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/benefits-of-active-etfs.html
+[Internal research]
+2. Selectors say 'ETF' and 'passive' were synonymous for years — definitions are still fluid; 56% would accept tracking error above 2%, signalling appetite for genuinely active ETFs — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Section 5, slides 12–14 and 50–53
+[External]
+3. The case for active ETFs vs index-tracking ETFs — Aberdeen Investments, “Know Your ETFs: Why Active”
 https://www.aberdeeninvestments.com/en-us/investor/insights-and-research/know-your-etfs-why-active
-2. The cost trade-off: higher fees mean active ETFs must clear a higher bar, with fee/performance data – Morningstar
+4. The cost trade-off: higher fees mean active ETFs must clear a higher bar — Morningstar
 https://www.morningstar.com/funds/active-versus-passive-etfs-why-lower-fees-still-win
-3. How the active/passive distinction is becoming a spectrum (systematic active, factor strategies) – Morningstar
-https://www.morningstar.com/funds/how-line-between-active-passive-etfs-is-blurring
-4. What active and passive ETFs share (the wrapper) and where they diverge (the strategy) – J.P. Morgan Asset Management, “ETFs Explained #1: Similarities of Active and Passive ETFs”
-https://am.jpmorgan.com/au/en/asset-management/adv/insights/investment-ideas/similarities-etfs/
-5. Balanced overview of the active vs passive trade-offs from the leading indexing provider – Vanguard, “Passive vs Active Investing: What's the Difference?”
-https://www3.vanguard.com.au/personal/learn/investment-options/active-vs-passive-investing</t>
+5. What active and passive ETFs share (the wrapper) and where they diverge (the strategy) — J.P. Morgan Asset Management
+https://am.jpmorgan.com/au/en/asset-management/adv/insights/investment-ideas/similarities-etfs/</t>
         </is>
       </c>
     </row>
@@ -648,18 +666,17 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>1. Manager selection risk / potential underperformance: share of active managers underperforming their benchmarks over 1–20 year horizons – S&amp;P Dow Jones Indices, SPIVA U.S. Scorecard
+          <t>[Internal research]
+1. Potential underperformance is the #1 perceived drawback (48%), then high management fees (30%), tracking error (23%) and complexity (18%); drawbacks broken down by client type — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Section 4 “Perceived benefits and drawbacks”, slides 15–16 and 48–49
+[External]
+2. Manager selection risk: share of active managers underperforming benchmarks over 1–20 year horizons — S&amp;P Dow Jones Indices, SPIVA U.S. Scorecard
 https://www.spglobal.com/spdji/en/spiva/article/spiva-us/
-2. Premiums and discounts to NAV: why they arise and what they mean for investors – Fidelity
+3. Premiums and discounts to NAV: why they arise and what they mean — Fidelity
 https://www.fidelity.com/learning-center/investment-products/etf/premiums-discounts-etfs
-3. Liquidity and trading concerns: price returns of some active ETFs lag their NAV returns because of trading frictions – Morningstar
+4. Liquidity/trading: price returns of some active ETFs lag NAV returns due to trading frictions — Morningstar
 https://www.morningstar.com/funds/you-might-not-always-get-returns-your-active-etf-earned
-4. Trading costs beyond the expense ratio (bid/ask spreads on active ETFs) – Morningstar
-https://www.morningstar.com/funds/your-active-etf-is-cheap-your-trade-might-not-be
-5. Whether active ETFs are inherently riskier than passive ETFs (risk depends on the underlying investments) – J.P. Morgan Asset Management, “Myth Busting #1”
-https://am.jpmorgan.com/sg/en/asset-management/adv/insights/portfolio-insights/etf-perspectives/active-etf-manual/myth-busting-active-etf-risks/
-6. Regulator's note that active funds typically carry higher costs and may underperform their index – U.S. SEC, Investor.gov
-https://www.investor.gov/introduction-investing/investing-basics/glossary/active-fund-actively-managed-fund</t>
+5. Whether active ETFs are inherently riskier than passive (risk depends on the underlying investments) — J.P. Morgan Asset Management, “Myth Busting #1”
+https://am.jpmorgan.com/sg/en/asset-management/adv/insights/portfolio-insights/etf-perspectives/active-etf-manual/myth-busting-active-etf-risks/</t>
         </is>
       </c>
     </row>
@@ -712,16 +729,20 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>1. How active ETFs are used to pursue specific objectives (income, total return, risk management, hard-to-reach markets) – Goldman Sachs Asset Management
+          <t>[Capital Group]
+1. “The benefits of active ETFs” — where manager judgement adds value: outperformance potential, downside protection, intraday flexibility
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/benefits-of-active-etfs.html
+2. Capital Group active ETF line-up by objective (core equity, income, international, fixed income) — matching strategy to investment objective
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds.html
+3. “Seeking to maximize tax efficiency with ETFs: 5 strategies” — concrete use cases for deploying active ETFs
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/5-ways-to-pursue-greater-tax-efficiency-with-etfs.html
+[Internal research]
+4. Main benefits selectors buy active ETFs for: potential outperformance (41%), low management fees (38%), niche/thematic access (38%), diversification, unique strategies — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Section 4, slide 15
+[External]
+5. How active ETFs are used to fine-tune portfolio construction — Goldman Sachs Asset Management
 https://am.gs.com/en-us/advisors/insights/article/2025/how-active-etfs-can-help-investors-fine-tune-portfolio-construction
-2. Whitepaper on active ETF categories and the manager's role in adding value – iShares/BlackRock, “Decoding Active ETFs”
-https://www.ishares.com/us/literature/whitepaper/decoding-active-etfs.pdf
-3. The case for active ETFs now – market conditions and strategy fit – Fidelity Institutional, “Why Active ETFs, Why Now?”
-https://institutional.fidelity.com/advisors/insights/topics/investing-ideas/why-active-etfs-why-now
-4. What advisors need to know about the rapid rise of active ETFs (42% of Q1 2026 net inflows) and where they fit – VettaFi via Advisor Perspectives
-https://www.advisorperspectives.com/commentaries/2026/02/11/what-advisors-need-to-know-about-the-rapid-rise-of-active-etfs
-5. Where manager judgement is designed to add value over an index – T. Rowe Price, “Active ETFs Designed to Outperform”
-https://www.troweprice.com/financial-intermediary/us/en/insights/articles/2021/q3/active-etfs-designed-to-outperform.html</t>
+6. Active ETF categories and the manager's role in adding value — iShares/BlackRock, “Decoding Active ETFs” (whitepaper)
+https://www.ishares.com/us/literature/whitepaper/decoding-active-etfs.pdf</t>
         </is>
       </c>
     </row>
@@ -746,16 +767,18 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>1. Practical advisor guidance on incorporating ETFs into client portfolios and matching them to client goals – Day Hagan Asset Management
-https://dayhagan.com/how-to-incorporate-etfs-into-client-portfolios
-2. Which active ETF categories advisors actually use and the client needs they map to (income, cash management, tax-efficient core) – The Daily Upside (Advisor)
+          <t>[Capital Group]
+1. Investment planning client-conversation tools — matching investment vehicles to client goals
+https://www.capitalgroup.com/advisor/tools/investment-planning.html
+2. Tax-sensitive clients as a natural active ETF audience — “5 strategies” tax-efficiency piece
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/5-ways-to-pursue-greater-tax-efficiency-with-etfs.html
+[Internal research]
+3. Openness to active ETFs by market and channel: wealth/investment managers most open, retail banks and insurance least; % of client portfolios where active ETFs are used; opportunity signals by segment — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Sections 2–3, slides 19 and 37–39
+[External]
+4. Which active ETF categories advisors use and the client needs they map to — The Daily Upside (Advisor)
 https://www.thedailyupside.com/advisor/investing-strategies/here-are-the-top-active-etfs-used-by-advisors/
-3. When advisors do (and don't) recommend active ETFs to clients – etf.com Advisor Center
-https://www.etf.com/sections/advisor-center/active-etf-financial-advisor-jpst-jaaa
-4. Advisor demand signal: 88% of advisors somewhat/very likely to increase active fixed income ETF allocations – VettaFi via Advisor Perspectives, “How Advisors Are Rewiring Fixed Income Portfolios”
-https://www.advisorperspectives.com/commentaries/2026/04/10/how-advisors-are-rewiring-fixed-income-portfolios
-5. Matching more conservative active ETF products to more conservative client profiles – ETF Trends, “Capital Group's Newer Active ETFs Offer More Conservative Approach”
-https://www.etftrends.com/capital-groups-newer-active-etfs-offer-more-conservative-approach/</t>
+5. Advisor demand signal: 88% of advisors likely to increase active fixed income ETF allocations — VettaFi via Advisor Perspectives
+https://www.advisorperspectives.com/commentaries/2026/04/10/how-advisors-are-rewiring-fixed-income-portfolios</t>
         </is>
       </c>
     </row>
@@ -779,22 +802,24 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>1. Research-based due diligence guide for active ETFs (people, process, price plus ETF-specific metrics) – Morningstar
+          <t>[Capital Group]
+1. ETF Insights &amp; Resources hub — evaluation and comparison materials for CG active ETFs
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources.html
+[Internal research]
+2. Where selectors research ETFs: asset manager websites (63%) and fund research/ratings agencies (61%) top the list; Morningstar, Bloomberg and JustETF are the preferred research sources — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Section 7 “ETF information sources”, slides 61–63
+[External]
+3. Morningstar's Guide to Active ETF Due Diligence (people, process, price + ETF-specific metrics)
 https://www.morningstar.com/business/insights/research/etf-due-diligence-guide
-2. Framework for active ETF due diligence combining fund-level and wrapper-level factors – John Hancock Investments
+4. Framework for active ETF due diligence — John Hancock Investments
 https://www.jhinvestments.com/resources/all-resources/business-building/etf-active-white-paper
-3. Qualitative + quantitative evaluation of active ETFs (philosophy, team, liquidity, spreads) – Goldman Sachs Asset Management
+5. Qualitative + quantitative evaluation of active ETFs — Goldman Sachs Asset Management, “Art and Science”
 https://am.gs.com/en-us/advisors/insights/article/2026/active-etf-due-diligence-combination-of-art-and-science
-4. Step-by-step checklist for comparing active ETF options across a peer group – Mackenzie Investments
-https://www.mackenzieinvestments.com/en/investments/by-type/etfs/etf-articles/your-step-by-step-guide-to-active-etf-due-diligence
-5. General ETF due diligence checklist (costs, liquidity, structure, issuer strength) – State Street Global Advisors
-https://www.ssga.com/us/en/intermediary/insights/a-etf-due-diligence-checklist
-6. Issuer framework for evaluating active ETFs across the peer group (PDF) – J.P. Morgan Asset Management, “Evaluating Active ETFs”
-https://am.jpmorgan.com/content/dam/jpm-am-aem/asiapacific/au/en/etf/evaluating-active-etf.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="375" customHeight="1">
+6. General ETF due diligence checklist — State Street Global Advisors
+https://www.ssga.com/us/en/intermediary/insights/a-etf-due-diligence-checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="409" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>How do I approach ETFs by client type?</t>
@@ -814,14 +839,20 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>1. Tailoring investment conversations to different client personas and their underlying beliefs – Morningstar
+          <t>[Capital Group]
+1. Chart stories — ready-made visuals for tailoring investment conversations to what each client cares about
+https://www.capitalgroup.com/advisor/pro/chart-stories.html
+2. “The power of storytelling” — using stories to land concepts with different client types (PracticeLab)
+https://www.capitalgroup.com/advisor/practicelab/articles/the-power-of-storytelling.html
+3. Investing-basics client conversation tools — talking points for foundational concepts
+https://www.capitalgroup.com/advisor/tools/investing-basics.html
+[Internal research]
+4. Four knowledge segments among intermediaries — Enthusiasm, Uncertainty, Education, Smart-beta confusion — with verbatim quotes per segment; maps directly onto the sheet's investor personas — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Section 2, slide 12
+[External]
+5. Tailoring conversations to different client personas and their underlying beliefs — Morningstar
 https://www.morningstar.com/financial-advisors/how-discuss-portfolio-diversification-with-different-types-clients
-2. Adapting communication style to client personality types when presenting recommendations – Brighthouse Financial, “A Guide to Speaking Your Client's Language”
-https://www.brighthousefinancial.com/content/dam/brighthouse-financial/protected/pdfs/shield/Guide-Speaking-Clients-Language.pdf
-3. Understanding the beliefs and concerns behind client resistance before responding – Hartford Funds
-https://www.hartfordfunds.com/insights/investor-insight/investor-behavior/your-money-story/how-to-respond-when-a-client-resists-recommendations.html
-4. The four most common misconceptions advisors will meet across client types, with rebuttals – J.P. Morgan Asset Management, “Active ETF Investing: Four Myths Debunked”
-https://am.jpmorgan.com/ca/en/asset-management/adv/funds/etf-perspectives/active-etf-investing-myths/</t>
+6. Understanding the beliefs behind client resistance before responding — Hartford Funds
+https://www.hartfordfunds.com/insights/investor-insight/investor-behavior/your-money-story/how-to-respond-when-a-client-resists-recommendations.html</t>
         </is>
       </c>
     </row>
@@ -873,16 +904,20 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>1. Advisor conversation-starter resources for opening investment discussions from the client's goals – BlackRock
+          <t>[Capital Group]
+1. Chart stories — visuals that open goal-based conversations an active ETF discussion can hang off
+https://www.capitalgroup.com/advisor/pro/chart-stories.html
+2. PracticeLab client-conversations topic hub — conversation starters and discovery techniques
+https://www.capitalgroup.com/advisor/ca/en/practicelab/topics/client-conversations.html
+3. “The power of storytelling” — engaging clients through stories rather than product pitches (PracticeLab)
+https://www.capitalgroup.com/advisor/practicelab/articles/the-power-of-storytelling.html
+[Internal research]
+4. The 5 stages of client decision-making around an innovation (knowledge/awareness → confirmation) and why education is the growth lever at the early-adopter stage; asset manager websites are selectors' #1 information source (63%) — advisors are the education channel — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Sections 1 and 7, slides 8 and 61
+[External]
+5. Advisor conversation starters for opening investment discussions from client goals — BlackRock
 https://www.blackrock.com/us/financial-professionals/resources/practice-management/conversation-starters
-2. Tools and talking points for structuring client conversations around goals and market events – Russell Investments, Client Conversation Center
-https://russellinvestments.com/content/ri/us/en/financial-professional/tools-and-education/business-solutions/client-conversation-center.html
-3. Framing the active ETF opportunity with clients (growth of the category and where it fits) – AllianceBernstein
-https://www.alliancebernstein.com/us/en-us/investments/etfs/etf-insights/actively-managed-etfs-are-on-the-move.html
-4. Current conversation hook: active ETFs took 42% of Q1 2026 net inflows and what that means for client portfolios – VettaFi via Advisor Perspectives
-https://www.advisorperspectives.com/commentaries/2026/02/11/what-advisors-need-to-know-about-the-rapid-rise-of-active-etfs
-5. How one issuer coaches advisors to pair active ETFs with client goals (accumulation vs decumulation) – ETF Database, “How Capital Group Shifted the Active ETF Playbook”
-https://etfdb.com/equity-etf-content-hub/capital-group-shifted-active-playbook/</t>
+6. Current conversation hook: active ETFs took 42% of Q1 2026 net inflows — VettaFi via Advisor Perspectives
+https://www.advisorperspectives.com/commentaries/2026/02/11/what-advisors-need-to-know-about-the-rapid-rise-of-active-etfs</t>
         </is>
       </c>
     </row>
@@ -909,18 +944,20 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>1. “What are active ETFs?” – Q&amp;A-format primer answering the most common first questions – HANetf
-https://hanetf.com/what-is-an-active-etf-your-questions-answered/
-2. “Why wouldn't I just index?” – data on active funds' struggle to beat index funds – CNBC
+          <t>[Capital Group]
+1. “Mythbusted: Active ETFs can be as tax efficient as passive ETFs” — answers the 'active can't be tax efficient / why not passive' objection with CG's own record
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/mythbusted-CG-capital-gains.html
+[Internal research]
+2. Verbatim client-style doubts to prepare for (“Is it a robot? Who's going to change the parameters?”, “these are complex and could require more intensive monitoring”); ranked drawbacks (underperformance 48%, fees 30%); tax and commission barriers by market — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Sections 2 and 4, slides 12 and 15–17
+[External]
+3. The four most common active ETF objections, each answered — J.P. Morgan Asset Management, “Four Myths Debunked”
+https://am.jpmorgan.com/ca/en/asset-management/adv/funds/etf-perspectives/active-etf-investing-myths/
+4. “Why wouldn't I just index?” — data on active funds' struggle to beat index funds — CNBC
 https://www.cnbc.com/2025/09/05/active-funds-struggle-to-beat-index-funds.html
-3. “Can active ETFs really outperform?” – whether outperformance persists – S&amp;P Dow Jones Indices, SPIVA Persistence Scorecard
+5. “Can active really outperform?” — persistence of outperformance — S&amp;P DJI, SPIVA Persistence Scorecard
 https://www.spglobal.com/spdji/en/spiva/article/us-persistence-scorecard/
-4. “Why should I pay more?” – fee differentials between active and passive ETFs – Morningstar
-https://www.morningstar.com/funds/active-versus-passive-etfs-why-lower-fees-still-win
-5. “Aren't active ETFs riskier than passive ones?” – risk depends on the underlying investments, not the management style – J.P. Morgan Asset Management, “Myth Busting #1”
-https://am.jpmorgan.com/sg/en/asset-management/adv/insights/portfolio-insights/etf-perspectives/active-etf-manual/myth-busting-active-etf-risks/
-6. The four most common active ETF objections in one place, each answered – J.P. Morgan Asset Management, “Active ETF Investing: Four Myths Debunked”
-https://am.jpmorgan.com/ca/en/asset-management/adv/funds/etf-perspectives/active-etf-investing-myths/</t>
+6. “Why should I pay more?” — fee differentials between active and passive ETFs — Morningstar
+https://www.morningstar.com/funds/active-versus-passive-etfs-why-lower-fees-still-win</t>
         </is>
       </c>
     </row>
@@ -945,23 +982,29 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>1. Using curiosity and empathy to uncover the belief behind an objection before reframing – Hartford Funds
-https://www.hartfordfunds.com/insights/investor-insight/investor-behavior/your-money-story/how-to-respond-when-a-client-resists-recommendations.html
-2. A repeatable framework for handling clients who reject recommendations while keeping the discussion on goals – Kitces.com
+          <t>[Capital Group]
+1. THE source for the four-box framework: “How to have better client conversations (even in uncertain times)” — Paul Cieslik's 4-Box Crucial Client Conversations model (acknowledge → perspective → confidence → opportunity), PracticeLab
+https://www.capitalgroup.com/advisor/practicelab/articles/have-better-client-conversations.html
+2. Chart stories — visual proof points to reframe objections during the conversation
+https://www.capitalgroup.com/advisor/pro/chart-stories.html
+3. Proof point vs active mutual fund: wrapper-driven tax efficiency (“Mythbusted”)
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/mythbusted-CG-capital-gains.html
+4. Proof point vs passive index: “The benefits of active ETFs” — outcomes and downside protection
+https://www.capitalgroup.com/advisor/investments/exchange-traded-funds/resources/benefits-of-active-etfs.html
+[Internal research]
+5. Reframing ammunition: outperformance is also the #1 perceived benefit (41%); ~50% of ETF users expect ETFs preferred to mutual funds vs 7% the reverse — RiF Active ETF Study — “Perceptions of Active ETFs in Europe” (EuroETF/EuroFSS, internal deck), Sections 3–4, slides 15 and 18
+[External]
+6. Handling clients who reject recommendations while keeping the discussion on goals — Kitces.com
 https://www.kitces.com/blog/163-michael-kitces-carl-richards-client-advice-implementation-recommendation-communication/
-3. Proof points for the active ETF wrapper vs active mutual funds and passive index funds (cost, tax efficiency, flexibility) – Fidelity Institutional
-https://institutional.fidelity.com/advisors/investment-solutions/strategies/active-etfs
-4. Ready-made rebuttals to the four most common objections (risk, liquidity, cost, performance) – J.P. Morgan Asset Management, “Active ETF Investing: Four Myths Debunked”
-https://am.jpmorgan.com/ca/en/asset-management/adv/funds/etf-perspectives/active-etf-investing-myths/
-5. Proof points vs passive: where active ETFs are designed to outperform and the evidence behind it – T. Rowe Price
-https://www.troweprice.com/financial-intermediary/us/en/insights/articles/2021/q3/active-etfs-designed-to-outperform.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
+7. Responding with curiosity and empathy when a client resists — Hartford Funds
+https://www.hartfordfunds.com/insights/investor-insight/investor-behavior/your-money-story/how-to-respond-when-a-client-resists-recommendations.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Yellow References cells were newly filled in (July 2026). White References cell (row 5, 'Why have active ETFs become so widespread?') keeps the original references; a URL was added to its previously link-less item 3.</t>
+          <t>References are grouped per cell: [Capital Group] = capitalgroup.com advisor/PracticeLab sources (incl. chart stories and the 4-Box client conversation framework); [Internal research] = RiF “Perceptions of Active ETFs in Europe” study (EuroETF/EuroFSS, private &amp; confidential deck — cite by section/slide, no public link); [External] = third-party sources. Yellow cells were filled/updated in this pass (July 2026); the white cell (row 5) keeps its original references with internal-deck and Capital Group items added.</t>
         </is>
       </c>
     </row>

</xml_diff>